<commit_message>
problem set 4 added, Raschka book chapters added
</commit_message>
<xml_diff>
--- a/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
+++ b/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viby\ecen45632_f26\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E91374A-11E7-415D-9A3D-ED076B3ECB97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF6CF7F-5517-465D-A874-9D51AC70365A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
+    <workbookView xWindow="788" yWindow="1823" windowWidth="19829" windowHeight="10649" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="40">
   <si>
     <t>ECEN 4/5632 Theory and Application of Digital Filters  Fall 2026</t>
   </si>
@@ -65,9 +65,6 @@
     <t>Week 6e</t>
   </si>
   <si>
-    <t>txt</t>
-  </si>
-  <si>
     <t>Lecture 1</t>
   </si>
   <si>
@@ -125,12 +122,6 @@
     <t>ipynb</t>
   </si>
   <si>
-    <t>PS 2</t>
-  </si>
-  <si>
-    <t>Q 1</t>
-  </si>
-  <si>
     <t>py</t>
   </si>
   <si>
@@ -150,6 +141,24 @@
   </si>
   <si>
     <t xml:space="preserve"> pptx, pdf, hc</t>
+  </si>
+  <si>
+    <t>PS 2, sol</t>
+  </si>
+  <si>
+    <t>Q2, sol</t>
+  </si>
+  <si>
+    <t>Q1, sol</t>
+  </si>
+  <si>
+    <t>#1</t>
+  </si>
+  <si>
+    <t>#2</t>
+  </si>
+  <si>
+    <t>PS3, sol</t>
   </si>
 </sst>
 </file>
@@ -539,34 +548,34 @@
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="C6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" t="s">
         <v>9</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" t="s">
+        <v>23</v>
+      </c>
+      <c r="J6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
-        <v>13</v>
-      </c>
-      <c r="G6" t="s">
-        <v>12</v>
-      </c>
-      <c r="H6" t="s">
-        <v>23</v>
-      </c>
-      <c r="I6" t="s">
+      <c r="K6" t="s">
         <v>24</v>
       </c>
-      <c r="J6" t="s">
-        <v>11</v>
-      </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>25</v>
-      </c>
-      <c r="L6" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.45">
@@ -574,28 +583,31 @@
         <v>2</v>
       </c>
       <c r="C8" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G8" t="s">
+        <v>30</v>
+      </c>
+      <c r="H8" t="s">
+        <v>31</v>
+      </c>
+      <c r="J8" t="s">
         <v>32</v>
       </c>
-      <c r="D8" t="s">
-        <v>31</v>
-      </c>
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" t="s">
-        <v>33</v>
-      </c>
-      <c r="G8" t="s">
-        <v>33</v>
-      </c>
-      <c r="H8" t="s">
-        <v>34</v>
-      </c>
-      <c r="J8" t="s">
-        <v>35</v>
-      </c>
       <c r="K8" t="s">
-        <v>29</v>
+        <v>36</v>
+      </c>
+      <c r="L8" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.45">
@@ -603,28 +615,34 @@
         <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D10" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" t="s">
+        <v>30</v>
+      </c>
+      <c r="G10" t="s">
+        <v>30</v>
+      </c>
+      <c r="H10" t="s">
         <v>31</v>
       </c>
-      <c r="F10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" t="s">
-        <v>33</v>
-      </c>
-      <c r="H10" t="s">
+      <c r="I10" t="s">
+        <v>26</v>
+      </c>
+      <c r="J10" t="s">
         <v>34</v>
       </c>
-      <c r="I10" t="s">
-        <v>27</v>
-      </c>
-      <c r="J10" t="s">
-        <v>28</v>
+      <c r="K10" t="s">
+        <v>35</v>
+      </c>
+      <c r="L10" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.45">
@@ -632,25 +650,28 @@
         <v>4</v>
       </c>
       <c r="C12" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" t="s">
+        <v>30</v>
+      </c>
+      <c r="G12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" t="s">
         <v>31</v>
       </c>
-      <c r="E12" t="s">
-        <v>31</v>
-      </c>
-      <c r="F12" t="s">
-        <v>33</v>
-      </c>
-      <c r="G12" t="s">
-        <v>33</v>
-      </c>
-      <c r="H12" t="s">
-        <v>34</v>
-      </c>
       <c r="I12" t="s">
-        <v>27</v>
+        <v>26</v>
+      </c>
+      <c r="J12" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
@@ -658,25 +679,25 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F14" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G14" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H14" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I14" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
@@ -684,70 +705,100 @@
         <v>6</v>
       </c>
       <c r="C16" t="s">
-        <v>8</v>
+        <v>29</v>
+      </c>
+      <c r="D16" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" t="s">
+        <v>30</v>
+      </c>
+      <c r="G16" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>7</v>
       </c>
+      <c r="C18" t="s">
+        <v>29</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" t="s">
+        <v>28</v>
+      </c>
+      <c r="F18" t="s">
+        <v>30</v>
+      </c>
+      <c r="G18" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>15</v>
+        <v>14</v>
+      </c>
+      <c r="C20" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C28" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="F28" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="G28" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="H28" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C30" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C32" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added Lecture 8 and IIR filter demo notebook
</commit_message>
<xml_diff>
--- a/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
+++ b/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viby\ecen45632_f26\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2EF6CF7F-5517-465D-A874-9D51AC70365A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937C7844-3EE0-44E1-B402-9F9C1BEE4A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="788" yWindow="1823" windowWidth="19829" windowHeight="10649" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
+    <workbookView xWindow="1125" yWindow="2160" windowWidth="19830" windowHeight="10650" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="44">
   <si>
     <t>ECEN 4/5632 Theory and Application of Digital Filters  Fall 2026</t>
   </si>
@@ -159,6 +159,18 @@
   </si>
   <si>
     <t>PS3, sol</t>
+  </si>
+  <si>
+    <t>txt</t>
+  </si>
+  <si>
+    <t>Q3, sol</t>
+  </si>
+  <si>
+    <t>#3</t>
+  </si>
+  <si>
+    <t>PS4, sol</t>
   </si>
 </sst>
 </file>
@@ -673,6 +685,12 @@
       <c r="J12" t="s">
         <v>39</v>
       </c>
+      <c r="K12" t="s">
+        <v>41</v>
+      </c>
+      <c r="L12" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
@@ -699,6 +717,9 @@
       <c r="I14" t="s">
         <v>26</v>
       </c>
+      <c r="J14" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
@@ -747,15 +768,33 @@
       <c r="C20" t="s">
         <v>29</v>
       </c>
+      <c r="D20" t="s">
+        <v>28</v>
+      </c>
+      <c r="E20" t="s">
+        <v>28</v>
+      </c>
+      <c r="F20" t="s">
+        <v>30</v>
+      </c>
+      <c r="G20" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>15</v>
       </c>
+      <c r="C22" t="s">
+        <v>40</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>16</v>
+      </c>
+      <c r="C24" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
Week05e demos and Lecture 9 updated
</commit_message>
<xml_diff>
--- a/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
+++ b/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viby\ecen45632_f26\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{937C7844-3EE0-44E1-B402-9F9C1BEE4A34}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED72874-E952-49B7-8B97-4521347AF92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1125" yWindow="2160" windowWidth="19830" windowHeight="10650" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="44">
   <si>
     <t>ECEN 4/5632 Theory and Application of Digital Filters  Fall 2026</t>
   </si>
@@ -161,9 +162,6 @@
     <t>PS3, sol</t>
   </si>
   <si>
-    <t>txt</t>
-  </si>
-  <si>
     <t>Q3, sol</t>
   </si>
   <si>
@@ -171,6 +169,9 @@
   </si>
   <si>
     <t>PS4, sol</t>
+  </si>
+  <si>
+    <t>txt, pf, hc</t>
   </si>
 </sst>
 </file>
@@ -686,10 +687,10 @@
         <v>39</v>
       </c>
       <c r="K12" t="s">
+        <v>40</v>
+      </c>
+      <c r="L12" t="s">
         <v>41</v>
-      </c>
-      <c r="L12" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.45">
@@ -718,7 +719,7 @@
         <v>26</v>
       </c>
       <c r="J14" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.45">
@@ -786,7 +787,13 @@
         <v>15</v>
       </c>
       <c r="C22" t="s">
-        <v>40</v>
+        <v>43</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
updated lectures 10 and 11, completed PS06 problem 1 solution
</commit_message>
<xml_diff>
--- a/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
+++ b/syllabus/ECEN45632_F26_CourseMaterialsInventory.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\viby\ecen45632_f26\syllabus\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ED72874-E952-49B7-8B97-4521347AF92B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CC0A1AD-F4EA-4F38-9492-24A66C3593CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" xr2:uid="{BF6D2AD3-84C2-4863-A168-54A8E33BD710}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="44">
   <si>
     <t>ECEN 4/5632 Theory and Application of Digital Filters  Fall 2026</t>
   </si>
@@ -795,6 +794,12 @@
       <c r="E22" t="s">
         <v>28</v>
       </c>
+      <c r="F22" t="s">
+        <v>30</v>
+      </c>
+      <c r="G22" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
@@ -803,10 +808,37 @@
       <c r="C24" t="s">
         <v>29</v>
       </c>
+      <c r="D24" t="s">
+        <v>28</v>
+      </c>
+      <c r="E24" t="s">
+        <v>28</v>
+      </c>
+      <c r="F24" t="s">
+        <v>30</v>
+      </c>
+      <c r="G24" t="s">
+        <v>30</v>
+      </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>17</v>
+      </c>
+      <c r="C26" t="s">
+        <v>29</v>
+      </c>
+      <c r="D26" t="s">
+        <v>28</v>
+      </c>
+      <c r="E26" t="s">
+        <v>28</v>
+      </c>
+      <c r="F26" t="s">
+        <v>30</v>
+      </c>
+      <c r="G26" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.45">

</xml_diff>